<commit_message>
Team Schedule Capture as of 10/17/2026 7:25 AM
</commit_message>
<xml_diff>
--- a/data/2026/cjsl/fall/brooklyn-city-fc-b14-15-blue.xlsx
+++ b/data/2026/cjsl/fall/brooklyn-city-fc-b14-15-blue.xlsx
@@ -71,12 +71,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" width="7.700000000000001"/>
-    <col min="2" max="2" bestFit="1" customWidth="1" width="27.500000000000004"/>
+    <col min="2" max="2" bestFit="1" customWidth="1" width="28.6"/>
     <col min="3" max="3" bestFit="1" customWidth="1" width="13.200000000000001"/>
     <col min="4" max="4" bestFit="1" customWidth="1" width="41.800000000000004"/>
     <col min="5" max="5" bestFit="1" customWidth="1" width="7.700000000000001"/>
     <col min="6" max="6" bestFit="1" customWidth="1" width="41.800000000000004"/>
-    <col min="7" max="7" bestFit="1" customWidth="1" width="48.400000000000006"/>
+    <col min="7" max="7" bestFit="1" customWidth="1" width="47.300000000000004"/>
     <col min="8" max="8" bestFit="1" customWidth="1" width="20.900000000000002"/>
     <col min="9" max="9" bestFit="1" customWidth="1" width="12.100000000000001"/>
   </cols>
@@ -175,36 +175,36 @@
     </row>
     <row r="3">
       <c r="A3" s="0" t="n">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Saturday, September 26, 2026</t>
+          <t>Saturday, October  3, 2026</t>
         </is>
       </c>
       <c r="C3" s="0" t="inlineStr">
         <is>
-          <t>16:00 EDT</t>
+          <t>15:00 EDT</t>
         </is>
       </c>
       <c r="D3" s="0" t="inlineStr">
         <is>
-          <t>Soccer Fun for Kids / Brooklyn Patriots 2014-2015 White</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="E3" s="0" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1 - 3</t>
         </is>
       </c>
       <c r="F3" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>FA Euro New York 2014/2015 Pre-MLS III</t>
         </is>
       </c>
       <c r="G3" s="0" t="inlineStr">
         <is>
-          <t>Prospect Park Parade Grounds Field 10B - Parade Grounds Field 10B</t>
+          <t>Bush Terminal Piers Park - Soccer 2A - small sided</t>
         </is>
       </c>
       <c r="H3" s="0" t="inlineStr">
@@ -214,42 +214,42 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t>Rained Out</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="n">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Saturday, October  3, 2026</t>
+          <t>Sunday, October 18, 2026</t>
         </is>
       </c>
       <c r="C4" s="0" t="inlineStr">
         <is>
-          <t>15:00 EDT</t>
+          <t>16:05 EDT</t>
         </is>
       </c>
       <c r="D4" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>DV7 NY B2014/15</t>
         </is>
       </c>
       <c r="E4" s="0" t="inlineStr">
         <is>
-          <t>1 - 3</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
         <is>
-          <t>FA Euro New York 2014/2015 Pre-MLS III</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="G4" s="0" t="inlineStr">
         <is>
-          <t>Bush Terminal Piers Park - Soccer 2A - small sided</t>
+          <t>Juniper Park - Field A (7v7)</t>
         </is>
       </c>
       <c r="H4" s="0" t="inlineStr">
@@ -265,21 +265,21 @@
     </row>
     <row r="5">
       <c r="A5" s="0" t="n">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Sunday, October 18, 2026</t>
+          <t>Saturday, October 24, 2026</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>16:05 EDT</t>
+          <t>15:45 EDT</t>
         </is>
       </c>
       <c r="D5" s="0" t="inlineStr">
         <is>
-          <t>DV7 NY B2014/15</t>
+          <t>SkillsU FC U12</t>
         </is>
       </c>
       <c r="E5" s="0" t="inlineStr">
@@ -294,7 +294,7 @@
       </c>
       <c r="G5" s="0" t="inlineStr">
         <is>
-          <t>Juniper Park - Field A (7v7)</t>
+          <t>Shore Road Park - Turf - Soccer Turf - Field 02</t>
         </is>
       </c>
       <c r="H5" s="0" t="inlineStr">
@@ -304,17 +304,17 @@
       </c>
       <c r="I5" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Scheduled</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="n">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Saturday, October 24, 2026</t>
+          <t>Saturday, October 31, 2026</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
@@ -324,7 +324,7 @@
       </c>
       <c r="D6" s="0" t="inlineStr">
         <is>
-          <t>SkillsU FC U12</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="E6" s="0" t="inlineStr">
@@ -334,12 +334,12 @@
       </c>
       <c r="F6" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>Soccer Fun for Kids / Brooklyn Patriots 2014-2015 White</t>
         </is>
       </c>
       <c r="G6" s="0" t="inlineStr">
         <is>
-          <t>Shore Road Park - Turf - Soccer Turf - Field 02</t>
+          <t>Red Hook Ball Fields - Field #8 9V9</t>
         </is>
       </c>
       <c r="H6" s="0" t="inlineStr">
@@ -349,27 +349,27 @@
       </c>
       <c r="I6" s="0" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="n">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Saturday, October 31, 2026</t>
+          <t>Saturday, November  7, 2026</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>15:45 EDT</t>
+          <t>19:45 EST</t>
         </is>
       </c>
       <c r="D7" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>FA Euro New York 2014/2015 Pre-MLS III</t>
         </is>
       </c>
       <c r="E7" s="0" t="inlineStr">
@@ -379,12 +379,12 @@
       </c>
       <c r="F7" s="0" t="inlineStr">
         <is>
-          <t>Soccer Fun for Kids / Brooklyn Patriots 2014-2015 White</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="G7" s="0" t="inlineStr">
         <is>
-          <t>Red Hook Ball Fields - Field #8 9V9</t>
+          <t>New Utrecht High School - Turf Field</t>
         </is>
       </c>
       <c r="H7" s="0" t="inlineStr">
@@ -394,27 +394,27 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Rescheduled</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="n">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>Saturday, November  7, 2026</t>
+          <t>Saturday, November 14, 2026</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>19:45 EST</t>
+          <t>14:15 EST</t>
         </is>
       </c>
       <c r="D8" s="0" t="inlineStr">
         <is>
-          <t>FA Euro New York 2014/2015 Pre-MLS III</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="E8" s="0" t="inlineStr">
@@ -424,12 +424,12 @@
       </c>
       <c r="F8" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>DV7 NY B2014/15</t>
         </is>
       </c>
       <c r="G8" s="0" t="inlineStr">
         <is>
-          <t>New Utrecht High School - Turf Field</t>
+          <t>Red Hook Park - Field 8 9v9 </t>
         </is>
       </c>
       <c r="H8" s="0" t="inlineStr">
@@ -439,27 +439,27 @@
       </c>
       <c r="I8" s="0" t="inlineStr">
         <is>
-          <t>Rescheduled</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="n">
-        <v>390</v>
+        <v>373</v>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Saturday, November 14, 2026</t>
+          <t>Sunday, November 15, 2026</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
-          <t>14:15 EST</t>
+          <t>13:30 EST</t>
         </is>
       </c>
       <c r="D9" s="0" t="inlineStr">
         <is>
-          <t>Brooklyn City FC F.C. B14/15 Blue</t>
+          <t>Soccer Fun for Kids / Brooklyn Patriots 2014-2015 White</t>
         </is>
       </c>
       <c r="E9" s="0" t="inlineStr">
@@ -469,12 +469,12 @@
       </c>
       <c r="F9" s="0" t="inlineStr">
         <is>
-          <t>DV7 NY B2014/15</t>
+          <t>Brooklyn City FC F.C. B14/15 Blue</t>
         </is>
       </c>
       <c r="G9" s="0" t="inlineStr">
         <is>
-          <t>Red Hook Park - Field 8 9v9 </t>
+          <t>Prospect Park, Parade Grounds Field 7B - Parade Grounds Field 7B</t>
         </is>
       </c>
       <c r="H9" s="0" t="inlineStr">
@@ -484,7 +484,7 @@
       </c>
       <c r="I9" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Rescheduled</t>
         </is>
       </c>
     </row>

</xml_diff>